<commit_message>
Added new page for simulation
</commit_message>
<xml_diff>
--- a/CasesAFR/AFR1.2.xlsx
+++ b/CasesAFR/AFR1.2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\s202180910\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\afsalem\Documents\GitHub\Senior_Project_Dashboard\CasesAFR\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FDC320A4-45A3-421C-B15D-E36DDD012061}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E848BCD1-CFAE-4F57-8C2B-B453C921CB1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Energy Streams" sheetId="1" r:id="rId1"/>
@@ -18,8 +18,17 @@
     <sheet name="Material Streams" sheetId="3" r:id="rId3"/>
     <sheet name="WorkBook Summary" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
     </ext>
@@ -28,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="45">
   <si>
     <t>Unit</t>
   </si>
@@ -160,12 +169,15 @@
   </si>
   <si>
     <t>Current Flowsheet Environment:</t>
+  </si>
+  <si>
+    <t>CO (ppm)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1033,15 +1045,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="21" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="16384" width="9.140625" style="1"/>
+    <col min="2" max="16384" width="9.1796875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1052,7 +1064,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -1072,508 +1084,475 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:J16"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="21" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.140625" style="1"/>
-    <col min="3" max="3" width="9.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.1796875" style="1"/>
+    <col min="3" max="3" width="9.26953125" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="12" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.26953125" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.26953125" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="12" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.26953125" style="1" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="12" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="16384" width="9.140625" style="1"/>
+    <col min="12" max="16384" width="9.1796875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B1" s="2" t="s">
-        <v>0</v>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B1" s="3" t="s">
+        <v>5</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="K1" s="3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3" s="4">
-        <v>0</v>
+      <c r="B3" s="4">
+        <v>0</v>
+      </c>
+      <c r="C3" s="1">
+        <v>2.1990886559466858E-20</v>
       </c>
       <c r="D3" s="1">
         <v>2.1990886559466858E-20</v>
       </c>
       <c r="E3" s="1">
+        <v>0</v>
+      </c>
+      <c r="F3" s="1">
         <v>2.1990886559466858E-20</v>
       </c>
-      <c r="F3" s="1">
-        <v>0</v>
-      </c>
-      <c r="G3" s="1">
+      <c r="G3" s="4">
+        <v>0.8</v>
+      </c>
+      <c r="H3" s="1">
+        <v>2.1990886559466855E-20</v>
+      </c>
+      <c r="I3" s="1">
+        <v>0.8</v>
+      </c>
+      <c r="J3" s="1">
         <v>2.1990886559466858E-20</v>
       </c>
-      <c r="H3" s="4">
-        <v>0.8</v>
-      </c>
-      <c r="I3" s="1">
-        <v>2.1990886559466855E-20</v>
-      </c>
-      <c r="J3" s="1">
-        <v>0.8</v>
-      </c>
-      <c r="K3" s="1">
-        <v>2.1990886559466858E-20</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" s="4">
-        <v>0</v>
+      <c r="B4" s="4">
+        <v>0</v>
+      </c>
+      <c r="C4" s="1">
+        <v>7.0121719166471783E-39</v>
       </c>
       <c r="D4" s="1">
         <v>7.0121719166471783E-39</v>
       </c>
       <c r="E4" s="1">
+        <v>0</v>
+      </c>
+      <c r="F4" s="1">
         <v>7.0121719166471783E-39</v>
       </c>
-      <c r="F4" s="1">
-        <v>0</v>
-      </c>
-      <c r="G4" s="1">
+      <c r="G4" s="4">
+        <v>0.1</v>
+      </c>
+      <c r="H4" s="1">
         <v>7.0121719166471783E-39</v>
       </c>
-      <c r="H4" s="4">
+      <c r="I4" s="1">
         <v>0.1</v>
       </c>
-      <c r="I4" s="1">
+      <c r="J4" s="1">
         <v>7.0121719166471783E-39</v>
       </c>
-      <c r="J4" s="1">
-        <v>0.1</v>
-      </c>
-      <c r="K4" s="1">
-        <v>7.0121719166471783E-39</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" s="4">
-        <v>0</v>
+      <c r="B5" s="4">
+        <v>0</v>
+      </c>
+      <c r="C5" s="1">
+        <v>7.4473971966515166E-42</v>
       </c>
       <c r="D5" s="1">
         <v>7.4473971966515166E-42</v>
       </c>
       <c r="E5" s="1">
+        <v>0</v>
+      </c>
+      <c r="F5" s="1">
         <v>7.4473971966515166E-42</v>
       </c>
-      <c r="F5" s="1">
-        <v>0</v>
-      </c>
-      <c r="G5" s="1">
+      <c r="G5" s="4">
+        <v>0.02</v>
+      </c>
+      <c r="H5" s="1">
         <v>7.4473971966515166E-42</v>
       </c>
-      <c r="H5" s="4">
+      <c r="I5" s="1">
         <v>0.02</v>
       </c>
-      <c r="I5" s="1">
+      <c r="J5" s="1">
         <v>7.4473971966515166E-42</v>
       </c>
-      <c r="J5" s="1">
-        <v>0.02</v>
-      </c>
-      <c r="K5" s="1">
-        <v>7.4473971966515166E-42</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" s="4">
-        <v>0</v>
+      <c r="B6" s="4">
+        <v>0</v>
+      </c>
+      <c r="C6" s="1">
+        <v>4.5921205107157199E-39</v>
       </c>
       <c r="D6" s="1">
         <v>4.5921205107157199E-39</v>
       </c>
       <c r="E6" s="1">
+        <v>0</v>
+      </c>
+      <c r="F6" s="1">
         <v>4.5921205107157199E-39</v>
       </c>
-      <c r="F6" s="1">
-        <v>0</v>
-      </c>
-      <c r="G6" s="1">
+      <c r="G6" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="H6" s="1">
         <v>4.5921205107157199E-39</v>
       </c>
-      <c r="H6" s="4">
+      <c r="I6" s="1">
         <v>0.01</v>
       </c>
-      <c r="I6" s="1">
+      <c r="J6" s="1">
         <v>4.5921205107157199E-39</v>
       </c>
-      <c r="J6" s="1">
-        <v>0.01</v>
-      </c>
-      <c r="K6" s="1">
-        <v>4.5921205107157199E-39</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C7" s="4">
-        <v>0</v>
+      <c r="B7" s="4">
+        <v>0</v>
+      </c>
+      <c r="C7" s="1">
+        <v>1.1715312351536785E-38</v>
       </c>
       <c r="D7" s="1">
         <v>1.1715312351536785E-38</v>
       </c>
       <c r="E7" s="1">
+        <v>0</v>
+      </c>
+      <c r="F7" s="1">
         <v>1.1715312351536785E-38</v>
       </c>
-      <c r="F7" s="1">
-        <v>0</v>
-      </c>
-      <c r="G7" s="1">
+      <c r="G7" s="4">
+        <v>0.05</v>
+      </c>
+      <c r="H7" s="1">
         <v>1.1715312351536785E-38</v>
       </c>
-      <c r="H7" s="4">
+      <c r="I7" s="1">
         <v>0.05</v>
       </c>
-      <c r="I7" s="1">
+      <c r="J7" s="1">
         <v>1.1715312351536785E-38</v>
       </c>
-      <c r="J7" s="1">
-        <v>0.05</v>
-      </c>
-      <c r="K7" s="1">
-        <v>1.1715312351536785E-38</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C8" s="4">
-        <v>0</v>
+      <c r="B8" s="4">
+        <v>0</v>
+      </c>
+      <c r="C8" s="1">
+        <v>4.2844854017893972E-4</v>
       </c>
       <c r="D8" s="1">
         <v>4.2844854017893972E-4</v>
       </c>
       <c r="E8" s="1">
+        <v>0</v>
+      </c>
+      <c r="F8" s="1">
         <v>4.2844854017893972E-4</v>
       </c>
-      <c r="F8" s="1">
-        <v>0</v>
-      </c>
-      <c r="G8" s="1">
+      <c r="G8" s="4">
+        <v>0</v>
+      </c>
+      <c r="H8" s="1">
         <v>4.2844854017893972E-4</v>
       </c>
-      <c r="H8" s="4">
-        <v>0</v>
-      </c>
       <c r="I8" s="1">
+        <v>0</v>
+      </c>
+      <c r="J8" s="1">
         <v>4.2844854017893972E-4</v>
       </c>
-      <c r="J8" s="1">
-        <v>0</v>
-      </c>
-      <c r="K8" s="1">
-        <v>4.2844854017893972E-4</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C9" s="4">
-        <v>0</v>
+      <c r="B9" s="4">
+        <v>0</v>
+      </c>
+      <c r="C9" s="1">
+        <v>8.6245606985092496E-2</v>
       </c>
       <c r="D9" s="1">
         <v>8.6245606985092496E-2</v>
       </c>
       <c r="E9" s="1">
+        <v>0</v>
+      </c>
+      <c r="F9" s="1">
         <v>8.6245606985092496E-2</v>
       </c>
-      <c r="F9" s="1">
-        <v>0</v>
-      </c>
-      <c r="G9" s="1">
+      <c r="G9" s="4">
+        <v>0</v>
+      </c>
+      <c r="H9" s="1">
+        <v>8.6245606985092482E-2</v>
+      </c>
+      <c r="I9" s="1">
+        <v>0</v>
+      </c>
+      <c r="J9" s="1">
         <v>8.6245606985092496E-2</v>
       </c>
-      <c r="H9" s="4">
-        <v>0</v>
-      </c>
-      <c r="I9" s="1">
-        <v>8.6245606985092482E-2</v>
-      </c>
-      <c r="J9" s="1">
-        <v>0</v>
-      </c>
-      <c r="K9" s="1">
-        <v>8.6245606985092496E-2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B10" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C10" s="4">
-        <v>0</v>
+      <c r="B10" s="4">
+        <v>0</v>
+      </c>
+      <c r="C10" s="1">
+        <v>0.1511957299977181</v>
       </c>
       <c r="D10" s="1">
         <v>0.1511957299977181</v>
       </c>
       <c r="E10" s="1">
+        <v>0</v>
+      </c>
+      <c r="F10" s="1">
         <v>0.1511957299977181</v>
       </c>
-      <c r="F10" s="1">
-        <v>0</v>
-      </c>
-      <c r="G10" s="1">
+      <c r="G10" s="4">
+        <v>0</v>
+      </c>
+      <c r="H10" s="1">
         <v>0.1511957299977181</v>
       </c>
-      <c r="H10" s="4">
-        <v>0</v>
-      </c>
       <c r="I10" s="1">
+        <v>0</v>
+      </c>
+      <c r="J10" s="1">
         <v>0.1511957299977181</v>
       </c>
-      <c r="J10" s="1">
-        <v>0</v>
-      </c>
-      <c r="K10" s="1">
-        <v>0.1511957299977181</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B11" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C11" s="4">
-        <v>0</v>
+      <c r="B11" s="4">
+        <v>0</v>
+      </c>
+      <c r="C11" s="1">
+        <v>1.6045651656187255E-4</v>
       </c>
       <c r="D11" s="1">
         <v>1.6045651656187255E-4</v>
       </c>
       <c r="E11" s="1">
+        <v>0</v>
+      </c>
+      <c r="F11" s="1">
         <v>1.6045651656187255E-4</v>
       </c>
-      <c r="F11" s="1">
-        <v>0</v>
-      </c>
-      <c r="G11" s="1">
+      <c r="G11" s="4">
+        <v>0.02</v>
+      </c>
+      <c r="H11" s="1">
         <v>1.6045651656187255E-4</v>
       </c>
-      <c r="H11" s="4">
+      <c r="I11" s="1">
         <v>0.02</v>
       </c>
-      <c r="I11" s="1">
+      <c r="J11" s="1">
         <v>1.6045651656187255E-4</v>
       </c>
-      <c r="J11" s="1">
-        <v>0.02</v>
-      </c>
-      <c r="K11" s="1">
-        <v>1.6045651656187255E-4</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B12" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C12" s="4">
-        <v>0</v>
+      <c r="B12" s="4">
+        <v>0</v>
+      </c>
+      <c r="C12" s="1">
+        <v>5.976971233829395E-6</v>
       </c>
       <c r="D12" s="1">
+        <v>5.9769712338293942E-6</v>
+      </c>
+      <c r="E12" s="1">
+        <v>0</v>
+      </c>
+      <c r="F12" s="1">
         <v>5.976971233829395E-6</v>
       </c>
-      <c r="E12" s="1">
+      <c r="G12" s="4">
+        <v>0</v>
+      </c>
+      <c r="H12" s="1">
+        <v>5.976971233829395E-6</v>
+      </c>
+      <c r="I12" s="1">
+        <v>0</v>
+      </c>
+      <c r="J12" s="1">
         <v>5.9769712338293942E-6</v>
       </c>
-      <c r="F12" s="1">
-        <v>0</v>
-      </c>
-      <c r="G12" s="1">
-        <v>5.976971233829395E-6</v>
-      </c>
-      <c r="H12" s="4">
-        <v>0</v>
-      </c>
-      <c r="I12" s="1">
-        <v>5.976971233829395E-6</v>
-      </c>
-      <c r="J12" s="1">
-        <v>0</v>
-      </c>
-      <c r="K12" s="1">
-        <v>5.9769712338293942E-6</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B13" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C13" s="4">
-        <v>0</v>
+      <c r="B13" s="4">
+        <v>0</v>
+      </c>
+      <c r="C13" s="1">
+        <v>3.6971728890678964E-3</v>
       </c>
       <c r="D13" s="1">
         <v>3.6971728890678964E-3</v>
       </c>
       <c r="E13" s="1">
+        <v>0</v>
+      </c>
+      <c r="F13" s="1">
         <v>3.6971728890678964E-3</v>
       </c>
-      <c r="F13" s="1">
-        <v>0</v>
-      </c>
-      <c r="G13" s="1">
+      <c r="G13" s="4">
+        <v>0</v>
+      </c>
+      <c r="H13" s="1">
         <v>3.6971728890678964E-3</v>
       </c>
-      <c r="H13" s="4">
-        <v>0</v>
-      </c>
       <c r="I13" s="1">
+        <v>0</v>
+      </c>
+      <c r="J13" s="1">
         <v>3.6971728890678964E-3</v>
       </c>
-      <c r="J13" s="1">
-        <v>0</v>
-      </c>
-      <c r="K13" s="1">
-        <v>3.6971728890678964E-3</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B14" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C14" s="4">
+      <c r="B14" s="4">
         <v>0.21</v>
+      </c>
+      <c r="C14" s="1">
+        <v>3.0134133297213657E-2</v>
       </c>
       <c r="D14" s="1">
         <v>3.0134133297213657E-2</v>
       </c>
       <c r="E14" s="1">
+        <v>0.21</v>
+      </c>
+      <c r="F14" s="1">
         <v>3.0134133297213657E-2</v>
       </c>
-      <c r="F14" s="1">
-        <v>0.21</v>
-      </c>
-      <c r="G14" s="1">
+      <c r="G14" s="4">
+        <v>0</v>
+      </c>
+      <c r="H14" s="1">
         <v>3.0134133297213657E-2</v>
       </c>
-      <c r="H14" s="4">
-        <v>0</v>
-      </c>
       <c r="I14" s="1">
+        <v>0</v>
+      </c>
+      <c r="J14" s="1">
         <v>3.0134133297213657E-2</v>
       </c>
-      <c r="J14" s="1">
-        <v>0</v>
-      </c>
-      <c r="K14" s="1">
-        <v>3.0134133297213657E-2</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B15" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C15" s="4">
+      <c r="B15" s="4">
         <v>0.79</v>
+      </c>
+      <c r="C15" s="1">
+        <v>0.72813247480293319</v>
       </c>
       <c r="D15" s="1">
         <v>0.72813247480293319</v>
       </c>
       <c r="E15" s="1">
+        <v>0.78999999999999992</v>
+      </c>
+      <c r="F15" s="1">
         <v>0.72813247480293319</v>
       </c>
-      <c r="F15" s="1">
-        <v>0.78999999999999992</v>
-      </c>
-      <c r="G15" s="1">
+      <c r="G15" s="4">
+        <v>0</v>
+      </c>
+      <c r="H15" s="1">
         <v>0.72813247480293319</v>
       </c>
-      <c r="H15" s="4">
-        <v>0</v>
-      </c>
       <c r="I15" s="1">
+        <v>0</v>
+      </c>
+      <c r="J15" s="1">
         <v>0.72813247480293319</v>
       </c>
-      <c r="J15" s="1">
-        <v>0</v>
-      </c>
-      <c r="K15" s="1">
-        <v>0.72813247480293319</v>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A16" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D16" s="1">
+        <f xml:space="preserve"> D8*(10^6)</f>
+        <v>428.44854017893971</v>
       </c>
     </row>
   </sheetData>
@@ -1582,22 +1561,22 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:K9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="21" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.140625" style="1"/>
-    <col min="3" max="3" width="9.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="11.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="9.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="11.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="16384" width="9.140625" style="1"/>
+    <col min="2" max="2" width="9.1796875" style="1"/>
+    <col min="3" max="3" width="9.26953125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="11.7265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="9.26953125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.7265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.26953125" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="11.7265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="16384" width="9.1796875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1629,7 +1608,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>28</v>
       </c>
@@ -1664,7 +1643,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>29</v>
       </c>
@@ -1699,7 +1678,7 @@
         <v>1554.6954361411294</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>31</v>
       </c>
@@ -1734,7 +1713,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>33</v>
       </c>
@@ -1769,7 +1748,7 @@
         <v>3152.6211175847347</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>35</v>
       </c>
@@ -1804,7 +1783,7 @@
         <v>88287.434076129764</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>37</v>
       </c>
@@ -1839,7 +1818,7 @@
         <v>110.4867626048072</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>3</v>
       </c>
@@ -1880,15 +1859,15 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="21" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="16384" width="9.140625" style="1"/>
+    <col min="2" max="16384" width="9.1796875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>39</v>
       </c>
@@ -1896,7 +1875,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
         <v>41</v>
       </c>
@@ -1904,7 +1883,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>43</v>
       </c>

</xml_diff>